<commit_message>
feat: complete Phase 1, 2, 3, and 4 with premium UI redesigns and dropdown selections
</commit_message>
<xml_diff>
--- a/public/templates/mau_sao_ke_ngan_hang.xlsx
+++ b/public/templates/mau_sao_ke_ngan_hang.xlsx
@@ -439,7 +439,7 @@
         <v>VCB2607010001</v>
       </c>
       <c r="D2" t="str">
-        <v>POS HCM ngay 01/07 - Tong hop giao dich the</v>
+        <v>POS HCM ngay 01/07 - doanh thu the tai quay</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -468,7 +468,7 @@
         <v>VCB2607010002</v>
       </c>
       <c r="D3" t="str">
-        <v>KH_ABC thanh toan cong no thang 06</v>
+        <v>KH_ABC thanh toan cong no dat tiec thang 06</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -497,7 +497,7 @@
         <v>VCB2607020001</v>
       </c>
       <c r="D4" t="str">
-        <v>Thanh toan NCC thuc pham sach</v>
+        <v>Thanh toan NCC nguyen lieu va bao bi</v>
       </c>
       <c r="E4">
         <v>18500000</v>
@@ -555,7 +555,7 @@
         <v>VCB2607030001</v>
       </c>
       <c r="D6" t="str">
-        <v>Vi dien tu doi soat doanh thu</v>
+        <v>Vi dien tu doi soat doanh thu delivery</v>
       </c>
       <c r="E6" t="str">
         <v/>

</xml_diff>

<commit_message>
feat: đối chiếu tiền vào, quyết toán ví có phí và duyệt phiếu hàng loạt
- Sao kê ngân hàng thêm cột "Loại thu/chi": phân loại ngay khi import, kiểm
  tra khoản mục đúng chiều tiền, hiện trên màn Đối soát.
- Tách phân loại thu/chi thành ba tầng theo cấu trúc P&L: Nhóm hạng mục P&L
  -> Hạng mục P&L -> Danh mục Thu/Chi.
- Phiếu thu/chi duyệt ngay khi lập; sửa trong ngày mở cho mọi vai trò có
  quyền sửa, qua ngày cần quyền mới edit_past. Thay nút duyệt từng dòng bằng
  ô chọn và nhóm thao tác duyệt/bỏ duyệt/xoá hàng loạt.
- Báo cáo Thu chi ngày thêm bảng đối chiếu tiền vào đã đủ chưa: thu ngân
  khai so với tiền thật đã về theo từng hình thức.
- Quyết toán ví/POS về ngân hàng: một phiếu ghi cả cộng tiền ngân hàng, xoá
  số treo ở ví và đẩy phần chênh sang chi phí quẹt thẻ trên P&L. Lập được
  ngay từ dòng sao kê ở màn Đối soát, kèm đánh dấu đã đối soát.
- Thanh bộ lọc/KPI dính như mini header ở các màn còn lại.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/mau_sao_ke_ngan_hang.xlsx
+++ b/public/templates/mau_sao_ke_ngan_hang.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +427,9 @@
       <c r="I1" t="str">
         <v>Goi y doi tac</v>
       </c>
+      <c r="J1" t="str">
+        <v>Loai thu/chi</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -456,6 +459,9 @@
       <c r="I2" t="str">
         <v>POS_HCM</v>
       </c>
+      <c r="J2" t="str">
+        <v>THU_BAN_HANG</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -485,6 +491,9 @@
       <c r="I3" t="str">
         <v>KH_ABC</v>
       </c>
+      <c r="J3" t="str">
+        <v>THU_BAN_HANG</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -514,6 +523,9 @@
       <c r="I4" t="str">
         <v>NCC_FOOD</v>
       </c>
+      <c r="J4" t="str">
+        <v>CHI_CONG_NO_NCC</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -543,6 +555,9 @@
       <c r="I5" t="str">
         <v>VCB</v>
       </c>
+      <c r="J5" t="str">
+        <v>CHI_PHI_NGAN_HANG</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -572,10 +587,13 @@
       <c r="I6" t="str">
         <v>WALLET_POS</v>
       </c>
+      <c r="J6" t="str">
+        <v>THU_BAN_HANG</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>